<commit_message>
Se agrega código de barras alterno en el 683
</commit_message>
<xml_diff>
--- a/posiciones_buscador.xlsx
+++ b/posiciones_buscador.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\desarrollos\buscador_posiciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC77DC0F-C466-4BCF-B0F5-B973C351A5F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3F1209B-6E85-4A5F-9DBB-B9E7607CFE66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{81345FCE-0991-44B1-AB97-4BC767A118BC}"/>
   </bookViews>
@@ -4193,9 +4193,6 @@
     <t>7501493889545</t>
   </si>
   <si>
-    <t>7503003406242, 7506346600308, 75968431605</t>
-  </si>
-  <si>
     <t>780083140205</t>
   </si>
   <si>
@@ -4671,6 +4668,9 @@
   </si>
   <si>
     <t>OMEGA 3,6,9, EPA/DHA CON ACEITE DE LINAZA Y OLIVO C/30</t>
+  </si>
+  <si>
+    <t>7503003406242, 7506346600308, 75968431605, 6650376816114</t>
   </si>
 </sst>
 </file>
@@ -16206,7 +16206,7 @@
         <v>7503003406242</v>
       </c>
       <c r="B477" s="1" t="s">
-        <v>1384</v>
+        <v>1543</v>
       </c>
       <c r="C477" s="2">
         <v>683</v>
@@ -16275,7 +16275,7 @@
         <v>780083139759</v>
       </c>
       <c r="B480" s="1" t="s">
-        <v>1385</v>
+        <v>1384</v>
       </c>
       <c r="C480" s="2">
         <v>687</v>
@@ -16298,7 +16298,7 @@
         <v>780083140212</v>
       </c>
       <c r="B481" s="1" t="s">
-        <v>1386</v>
+        <v>1385</v>
       </c>
       <c r="C481" s="2">
         <v>688</v>
@@ -16321,7 +16321,7 @@
         <v>7502009746215</v>
       </c>
       <c r="B482" s="1" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
       <c r="C482" s="2">
         <v>690</v>
@@ -16344,7 +16344,7 @@
         <v>7501349020962</v>
       </c>
       <c r="B483" s="1" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="C483" s="2">
         <v>692</v>
@@ -16367,7 +16367,7 @@
         <v>656599041216</v>
       </c>
       <c r="B484" s="1" t="s">
-        <v>1389</v>
+        <v>1388</v>
       </c>
       <c r="C484" s="2">
         <v>693</v>
@@ -16390,7 +16390,7 @@
         <v>785118753788</v>
       </c>
       <c r="B485" s="1" t="s">
-        <v>1390</v>
+        <v>1389</v>
       </c>
       <c r="C485" s="2">
         <v>694</v>
@@ -16459,7 +16459,7 @@
         <v>7503000422283</v>
       </c>
       <c r="B488" s="1" t="s">
-        <v>1391</v>
+        <v>1390</v>
       </c>
       <c r="C488" s="2">
         <v>698</v>
@@ -16482,7 +16482,7 @@
         <v>7501075715095</v>
       </c>
       <c r="B489" s="1" t="s">
-        <v>1392</v>
+        <v>1391</v>
       </c>
       <c r="C489" s="2">
         <v>699</v>
@@ -16505,7 +16505,7 @@
         <v>7501075715088</v>
       </c>
       <c r="B490" s="1" t="s">
-        <v>1393</v>
+        <v>1392</v>
       </c>
       <c r="C490" s="2">
         <v>700</v>
@@ -16528,7 +16528,7 @@
         <v>7501547522145</v>
       </c>
       <c r="B491" s="1" t="s">
-        <v>1394</v>
+        <v>1393</v>
       </c>
       <c r="C491" s="2">
         <v>701</v>
@@ -16574,7 +16574,7 @@
         <v>750200165441</v>
       </c>
       <c r="B493" s="1" t="s">
-        <v>1395</v>
+        <v>1394</v>
       </c>
       <c r="C493" s="2">
         <v>704</v>
@@ -16597,7 +16597,7 @@
         <v>7501471888249</v>
       </c>
       <c r="B494" s="1" t="s">
-        <v>1396</v>
+        <v>1395</v>
       </c>
       <c r="C494" s="2">
         <v>709</v>
@@ -16620,7 +16620,7 @@
         <v>7501258205078</v>
       </c>
       <c r="B495" s="1" t="s">
-        <v>1397</v>
+        <v>1396</v>
       </c>
       <c r="C495" s="2">
         <v>710</v>
@@ -16643,7 +16643,7 @@
         <v>7502216798786</v>
       </c>
       <c r="B496" s="1" t="s">
-        <v>1398</v>
+        <v>1397</v>
       </c>
       <c r="C496" s="2">
         <v>711</v>
@@ -16666,7 +16666,7 @@
         <v>7502211782483</v>
       </c>
       <c r="B497" s="1" t="s">
-        <v>1399</v>
+        <v>1398</v>
       </c>
       <c r="C497" s="2">
         <v>712</v>
@@ -16689,7 +16689,7 @@
         <v>780083148423</v>
       </c>
       <c r="B498" s="1" t="s">
-        <v>1400</v>
+        <v>1399</v>
       </c>
       <c r="C498" s="2">
         <v>713</v>
@@ -16735,7 +16735,7 @@
         <v>7502009744983</v>
       </c>
       <c r="B500" s="1" t="s">
-        <v>1401</v>
+        <v>1400</v>
       </c>
       <c r="C500" s="2">
         <v>716</v>
@@ -16758,7 +16758,7 @@
         <v>780083143565</v>
       </c>
       <c r="B501" s="1" t="s">
-        <v>1402</v>
+        <v>1401</v>
       </c>
       <c r="C501" s="2">
         <v>717</v>
@@ -16781,7 +16781,7 @@
         <v>7501075717686</v>
       </c>
       <c r="B502" s="1" t="s">
-        <v>1403</v>
+        <v>1402</v>
       </c>
       <c r="C502" s="2">
         <v>718</v>
@@ -16804,7 +16804,7 @@
         <v>7501349029170</v>
       </c>
       <c r="B503" s="1" t="s">
-        <v>1404</v>
+        <v>1403</v>
       </c>
       <c r="C503" s="2">
         <v>719</v>
@@ -16827,7 +16827,7 @@
         <v>7502216808614</v>
       </c>
       <c r="B504" s="1" t="s">
-        <v>1405</v>
+        <v>1404</v>
       </c>
       <c r="C504" s="2">
         <v>720</v>
@@ -16850,7 +16850,7 @@
         <v>7502216808645</v>
       </c>
       <c r="B505" s="1" t="s">
-        <v>1406</v>
+        <v>1405</v>
       </c>
       <c r="C505" s="2">
         <v>721</v>
@@ -16873,7 +16873,7 @@
         <v>75049812</v>
       </c>
       <c r="B506" s="1" t="s">
-        <v>1407</v>
+        <v>1406</v>
       </c>
       <c r="C506" s="2">
         <v>722</v>
@@ -16896,7 +16896,7 @@
         <v>7506022304452</v>
       </c>
       <c r="B507" s="1" t="s">
-        <v>1408</v>
+        <v>1407</v>
       </c>
       <c r="C507" s="2">
         <v>723</v>
@@ -16942,7 +16942,7 @@
         <v>729513107890</v>
       </c>
       <c r="B509" s="1" t="s">
-        <v>1409</v>
+        <v>1408</v>
       </c>
       <c r="C509" s="2">
         <v>727</v>
@@ -16965,7 +16965,7 @@
         <v>729513107944</v>
       </c>
       <c r="B510" s="1" t="s">
-        <v>1410</v>
+        <v>1409</v>
       </c>
       <c r="C510" s="2">
         <v>728</v>
@@ -16988,7 +16988,7 @@
         <v>780083140731</v>
       </c>
       <c r="B511" s="1" t="s">
-        <v>1411</v>
+        <v>1410</v>
       </c>
       <c r="C511" s="2">
         <v>729</v>
@@ -17011,7 +17011,7 @@
         <v>7501471889352</v>
       </c>
       <c r="B512" s="1" t="s">
-        <v>1412</v>
+        <v>1411</v>
       </c>
       <c r="C512" s="2">
         <v>730</v>
@@ -17034,7 +17034,7 @@
         <v>729513107906</v>
       </c>
       <c r="B513" s="1" t="s">
-        <v>1413</v>
+        <v>1412</v>
       </c>
       <c r="C513" s="2">
         <v>731</v>
@@ -17080,7 +17080,7 @@
         <v>7501289512633</v>
       </c>
       <c r="B515" s="1" t="s">
-        <v>1414</v>
+        <v>1413</v>
       </c>
       <c r="C515" s="2">
         <v>733</v>
@@ -17103,7 +17103,7 @@
         <v>7502004530079</v>
       </c>
       <c r="B516" s="1" t="s">
-        <v>1415</v>
+        <v>1414</v>
       </c>
       <c r="C516" s="2">
         <v>734</v>
@@ -17126,7 +17126,7 @@
         <v>729513107883</v>
       </c>
       <c r="B517" s="1" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
       <c r="C517" s="2">
         <v>735</v>
@@ -17149,7 +17149,7 @@
         <v>7503002773161</v>
       </c>
       <c r="B518" s="1" t="s">
-        <v>1417</v>
+        <v>1416</v>
       </c>
       <c r="C518" s="2">
         <v>737</v>
@@ -17172,7 +17172,7 @@
         <v>7501258206525</v>
       </c>
       <c r="B519" s="1" t="s">
-        <v>1418</v>
+        <v>1417</v>
       </c>
       <c r="C519" s="2">
         <v>739</v>
@@ -17195,7 +17195,7 @@
         <v>7501361111501</v>
       </c>
       <c r="B520" s="1" t="s">
-        <v>1419</v>
+        <v>1418</v>
       </c>
       <c r="C520" s="2">
         <v>740</v>
@@ -17218,7 +17218,7 @@
         <v>7502216803916</v>
       </c>
       <c r="B521" s="1" t="s">
-        <v>1420</v>
+        <v>1419</v>
       </c>
       <c r="C521" s="2">
         <v>742</v>
@@ -17241,7 +17241,7 @@
         <v>7702136645003</v>
       </c>
       <c r="B522" s="1" t="s">
-        <v>1421</v>
+        <v>1420</v>
       </c>
       <c r="C522" s="2">
         <v>744</v>
@@ -17264,7 +17264,7 @@
         <v>736211494979</v>
       </c>
       <c r="B523" s="1" t="s">
-        <v>1422</v>
+        <v>1421</v>
       </c>
       <c r="C523" s="2">
         <v>746</v>
@@ -17287,7 +17287,7 @@
         <v>785120754841</v>
       </c>
       <c r="B524" s="1" t="s">
-        <v>1423</v>
+        <v>1422</v>
       </c>
       <c r="C524" s="2">
         <v>747</v>
@@ -17310,7 +17310,7 @@
         <v>785120755046</v>
       </c>
       <c r="B525" s="1" t="s">
-        <v>1424</v>
+        <v>1423</v>
       </c>
       <c r="C525" s="2">
         <v>748</v>
@@ -17333,7 +17333,7 @@
         <v>785120755022</v>
       </c>
       <c r="B526" s="1" t="s">
-        <v>1425</v>
+        <v>1424</v>
       </c>
       <c r="C526" s="2">
         <v>749</v>
@@ -17356,7 +17356,7 @@
         <v>7501349025806</v>
       </c>
       <c r="B527" s="1" t="s">
-        <v>1426</v>
+        <v>1425</v>
       </c>
       <c r="C527" s="2">
         <v>751</v>
@@ -17379,7 +17379,7 @@
         <v>7501493888784</v>
       </c>
       <c r="B528" s="1" t="s">
-        <v>1427</v>
+        <v>1426</v>
       </c>
       <c r="C528" s="2">
         <v>752</v>
@@ -17402,7 +17402,7 @@
         <v>7502216797369</v>
       </c>
       <c r="B529" s="1" t="s">
-        <v>1428</v>
+        <v>1427</v>
       </c>
       <c r="C529" s="2">
         <v>753</v>
@@ -17448,7 +17448,7 @@
         <v>637420200897</v>
       </c>
       <c r="B531" s="1" t="s">
-        <v>1429</v>
+        <v>1428</v>
       </c>
       <c r="C531" s="2">
         <v>758</v>
@@ -17471,7 +17471,7 @@
         <v>7501250882024</v>
       </c>
       <c r="B532" s="1" t="s">
-        <v>1430</v>
+        <v>1429</v>
       </c>
       <c r="C532" s="2">
         <v>759</v>
@@ -17494,7 +17494,7 @@
         <v>7502009743986</v>
       </c>
       <c r="B533" s="1" t="s">
-        <v>1431</v>
+        <v>1430</v>
       </c>
       <c r="C533" s="2">
         <v>766</v>
@@ -17517,7 +17517,7 @@
         <v>7502009747168</v>
       </c>
       <c r="B534" s="1" t="s">
-        <v>1432</v>
+        <v>1431</v>
       </c>
       <c r="C534" s="2">
         <v>767</v>
@@ -17747,7 +17747,7 @@
         <v>729513100686</v>
       </c>
       <c r="B544" s="1" t="s">
-        <v>1433</v>
+        <v>1432</v>
       </c>
       <c r="C544" s="2">
         <v>780</v>
@@ -17793,7 +17793,7 @@
         <v>759684155017</v>
       </c>
       <c r="B546" s="1" t="s">
-        <v>1434</v>
+        <v>1433</v>
       </c>
       <c r="C546" s="2">
         <v>782</v>
@@ -17839,7 +17839,7 @@
         <v>759684351051</v>
       </c>
       <c r="B548" s="1" t="s">
-        <v>1435</v>
+        <v>1434</v>
       </c>
       <c r="C548" s="2">
         <v>789</v>
@@ -17862,7 +17862,7 @@
         <v>7503003406402</v>
       </c>
       <c r="B549" s="1" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="C549" s="2">
         <v>794</v>
@@ -17885,7 +17885,7 @@
         <v>759684432071</v>
       </c>
       <c r="B550" s="1" t="s">
-        <v>1437</v>
+        <v>1436</v>
       </c>
       <c r="C550" s="2">
         <v>795</v>
@@ -17908,7 +17908,7 @@
         <v>780083148843</v>
       </c>
       <c r="B551" s="1" t="s">
-        <v>1438</v>
+        <v>1437</v>
       </c>
       <c r="C551" s="2">
         <v>800</v>
@@ -17931,7 +17931,7 @@
         <v>780083146955</v>
       </c>
       <c r="B552" s="1" t="s">
-        <v>1439</v>
+        <v>1438</v>
       </c>
       <c r="C552" s="2">
         <v>803</v>
@@ -17954,7 +17954,7 @@
         <v>7501825305149</v>
       </c>
       <c r="B553" s="1" t="s">
-        <v>1440</v>
+        <v>1439</v>
       </c>
       <c r="C553" s="2">
         <v>804</v>
@@ -17977,7 +17977,7 @@
         <v>7502009747373</v>
       </c>
       <c r="B554" s="1" t="s">
-        <v>1441</v>
+        <v>1440</v>
       </c>
       <c r="C554" s="2">
         <v>811</v>
@@ -18046,7 +18046,7 @@
         <v>7502003389975</v>
       </c>
       <c r="B557" s="1" t="s">
-        <v>1442</v>
+        <v>1441</v>
       </c>
       <c r="C557" s="2">
         <v>826</v>
@@ -18115,7 +18115,7 @@
         <v>7502268542207</v>
       </c>
       <c r="B560" s="1" t="s">
-        <v>1443</v>
+        <v>1442</v>
       </c>
       <c r="C560" s="2">
         <v>831</v>
@@ -18161,7 +18161,7 @@
         <v>7502247373914</v>
       </c>
       <c r="B562" s="1" t="s">
-        <v>1444</v>
+        <v>1443</v>
       </c>
       <c r="C562" s="2">
         <v>835</v>
@@ -18437,7 +18437,7 @@
         <v>759684900105</v>
       </c>
       <c r="B574" s="1" t="s">
-        <v>1445</v>
+        <v>1444</v>
       </c>
       <c r="C574" s="2">
         <v>874</v>
@@ -18460,7 +18460,7 @@
         <v>759684311451</v>
       </c>
       <c r="B575" s="1" t="s">
-        <v>1446</v>
+        <v>1445</v>
       </c>
       <c r="C575" s="2">
         <v>875</v>
@@ -18506,7 +18506,7 @@
         <v>7501590286223</v>
       </c>
       <c r="B577" s="1" t="s">
-        <v>1447</v>
+        <v>1446</v>
       </c>
       <c r="C577" s="2">
         <v>878</v>
@@ -18552,7 +18552,7 @@
         <v>7501590284779</v>
       </c>
       <c r="B579" s="1" t="s">
-        <v>1448</v>
+        <v>1447</v>
       </c>
       <c r="C579" s="2">
         <v>881</v>
@@ -18621,7 +18621,7 @@
         <v>773042188775</v>
       </c>
       <c r="B582" s="1" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="C582" s="2">
         <v>884</v>
@@ -18759,7 +18759,7 @@
         <v>0</v>
       </c>
       <c r="B588" s="1" t="s">
-        <v>1450</v>
+        <v>1449</v>
       </c>
       <c r="C588" s="2">
         <v>893</v>
@@ -18782,7 +18782,7 @@
         <v>759684154034</v>
       </c>
       <c r="B589" s="1" t="s">
-        <v>1451</v>
+        <v>1450</v>
       </c>
       <c r="C589" s="2">
         <v>902</v>
@@ -18805,7 +18805,7 @@
         <v>7501109763375</v>
       </c>
       <c r="B590" s="1" t="s">
-        <v>1452</v>
+        <v>1451</v>
       </c>
       <c r="C590" s="2">
         <v>903</v>
@@ -18828,7 +18828,7 @@
         <v>7502216791619</v>
       </c>
       <c r="B591" s="1" t="s">
-        <v>1453</v>
+        <v>1452</v>
       </c>
       <c r="C591" s="2">
         <v>904</v>
@@ -18897,7 +18897,7 @@
         <v>7501349027060</v>
       </c>
       <c r="B594" s="1" t="s">
-        <v>1454</v>
+        <v>1453</v>
       </c>
       <c r="C594" s="2">
         <v>907</v>
@@ -18920,7 +18920,7 @@
         <v>7501349025059</v>
       </c>
       <c r="B595" s="1" t="s">
-        <v>1455</v>
+        <v>1454</v>
       </c>
       <c r="C595" s="2">
         <v>908</v>
@@ -19058,7 +19058,7 @@
         <v>7502227876398</v>
       </c>
       <c r="B601" s="1" t="s">
-        <v>1456</v>
+        <v>1455</v>
       </c>
       <c r="C601" s="2">
         <v>914</v>
@@ -19219,7 +19219,7 @@
         <v>7502216790896</v>
       </c>
       <c r="B608" s="1" t="s">
-        <v>1457</v>
+        <v>1456</v>
       </c>
       <c r="C608" s="2">
         <v>978</v>
@@ -19242,7 +19242,7 @@
         <v>821998000571</v>
       </c>
       <c r="B609" s="1" t="s">
-        <v>1458</v>
+        <v>1457</v>
       </c>
       <c r="C609" s="2">
         <v>979</v>
@@ -19587,7 +19587,7 @@
         <v>5601332</v>
       </c>
       <c r="B624" s="1" t="s">
-        <v>1459</v>
+        <v>1458</v>
       </c>
       <c r="C624" s="2">
         <v>1051</v>
@@ -19978,7 +19978,7 @@
         <v>7501349021624</v>
       </c>
       <c r="B641" s="1" t="s">
-        <v>1460</v>
+        <v>1459</v>
       </c>
       <c r="C641" s="2">
         <v>1115</v>
@@ -20599,7 +20599,7 @@
         <v>714908107098</v>
       </c>
       <c r="B668" s="1" t="s">
-        <v>1461</v>
+        <v>1460</v>
       </c>
       <c r="C668" s="2">
         <v>9002</v>
@@ -20668,7 +20668,7 @@
         <v>714908105483</v>
       </c>
       <c r="B671" s="1" t="s">
-        <v>1462</v>
+        <v>1461</v>
       </c>
       <c r="C671" s="2">
         <v>9009</v>
@@ -20691,7 +20691,7 @@
         <v>7501258206723</v>
       </c>
       <c r="B672" s="1" t="s">
-        <v>1463</v>
+        <v>1462</v>
       </c>
       <c r="C672" s="2">
         <v>9013</v>
@@ -20829,7 +20829,7 @@
         <v>7502214010415</v>
       </c>
       <c r="B678" s="1" t="s">
-        <v>1464</v>
+        <v>1463</v>
       </c>
       <c r="C678" s="2">
         <v>9021</v>
@@ -20921,7 +20921,7 @@
         <v>7502214011054</v>
       </c>
       <c r="B682" s="1" t="s">
-        <v>1465</v>
+        <v>1464</v>
       </c>
       <c r="C682" s="2">
         <v>9031</v>
@@ -20967,7 +20967,7 @@
         <v>7502214011030</v>
       </c>
       <c r="B684" s="1" t="s">
-        <v>1466</v>
+        <v>1465</v>
       </c>
       <c r="C684" s="2">
         <v>9033</v>
@@ -21036,7 +21036,7 @@
         <v>7502214010347</v>
       </c>
       <c r="B687" s="1" t="s">
-        <v>1467</v>
+        <v>1466</v>
       </c>
       <c r="C687" s="2">
         <v>9038</v>
@@ -21082,7 +21082,7 @@
         <v>75035000242</v>
       </c>
       <c r="B689" s="1" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
       <c r="C689" s="2">
         <v>9051</v>
@@ -21105,7 +21105,7 @@
         <v>7502244010126</v>
       </c>
       <c r="B690" s="1" t="s">
-        <v>1469</v>
+        <v>1468</v>
       </c>
       <c r="C690" s="2">
         <v>9054</v>
@@ -21220,7 +21220,7 @@
         <v>7503007662194</v>
       </c>
       <c r="B695" s="1" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="C695" s="2">
         <v>9069</v>
@@ -21243,7 +21243,7 @@
         <v>7503007662255</v>
       </c>
       <c r="B696" s="1" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="C696" s="2">
         <v>9070</v>
@@ -21312,7 +21312,7 @@
         <v>7502214011023</v>
       </c>
       <c r="B699" s="1" t="s">
-        <v>1472</v>
+        <v>1471</v>
       </c>
       <c r="C699" s="2">
         <v>9078</v>
@@ -21404,7 +21404,7 @@
         <v>7502010840193</v>
       </c>
       <c r="B703" s="1" t="s">
-        <v>1473</v>
+        <v>1472</v>
       </c>
       <c r="C703" s="2">
         <v>9086</v>
@@ -21427,7 +21427,7 @@
         <v>7503007202437</v>
       </c>
       <c r="B704" s="1" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
       <c r="C704" s="2">
         <v>9089</v>
@@ -21519,7 +21519,7 @@
         <v>803288480669</v>
       </c>
       <c r="B708" s="1" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="C708" s="2">
         <v>9107</v>
@@ -21542,7 +21542,7 @@
         <v>714908100099</v>
       </c>
       <c r="B709" s="1" t="s">
-        <v>1476</v>
+        <v>1475</v>
       </c>
       <c r="C709" s="2">
         <v>9108</v>
@@ -21634,7 +21634,7 @@
         <v>7502010840292</v>
       </c>
       <c r="B713" s="1" t="s">
-        <v>1477</v>
+        <v>1476</v>
       </c>
       <c r="C713" s="2">
         <v>9120</v>
@@ -21680,7 +21680,7 @@
         <v>7501384504939</v>
       </c>
       <c r="B715" s="1" t="s">
-        <v>1478</v>
+        <v>1477</v>
       </c>
       <c r="C715" s="2">
         <v>9137</v>
@@ -21703,7 +21703,7 @@
         <v>7501590283048</v>
       </c>
       <c r="B716" s="1" t="s">
-        <v>1479</v>
+        <v>1478</v>
       </c>
       <c r="C716" s="2">
         <v>9138</v>
@@ -21772,7 +21772,7 @@
         <v>714908100518</v>
       </c>
       <c r="B719" s="1" t="s">
-        <v>1480</v>
+        <v>1479</v>
       </c>
       <c r="C719" s="2">
         <v>9146</v>
@@ -21795,7 +21795,7 @@
         <v>7502009743993</v>
       </c>
       <c r="B720" s="1" t="s">
-        <v>1481</v>
+        <v>1480</v>
       </c>
       <c r="C720" s="2">
         <v>9147</v>
@@ -21933,7 +21933,7 @@
         <v>7503181042881</v>
       </c>
       <c r="B726" s="1" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
       <c r="C726" s="2">
         <v>9173</v>
@@ -22071,7 +22071,7 @@
         <v>7501075712223</v>
       </c>
       <c r="B732" s="1" t="s">
-        <v>1483</v>
+        <v>1482</v>
       </c>
       <c r="C732" s="2">
         <v>9193</v>
@@ -22094,7 +22094,7 @@
         <v>7500326106972</v>
       </c>
       <c r="B733" s="1" t="s">
-        <v>1484</v>
+        <v>1483</v>
       </c>
       <c r="C733" s="2">
         <v>9195</v>
@@ -22163,7 +22163,7 @@
         <v>7503008344150</v>
       </c>
       <c r="B736" s="1" t="s">
-        <v>1485</v>
+        <v>1484</v>
       </c>
       <c r="C736" s="2">
         <v>9199</v>
@@ -22278,7 +22278,7 @@
         <v>7502259891376</v>
       </c>
       <c r="B741" s="1" t="s">
-        <v>1486</v>
+        <v>1485</v>
       </c>
       <c r="C741" s="2">
         <v>9227</v>
@@ -22347,7 +22347,7 @@
         <v>7502259891079</v>
       </c>
       <c r="B744" s="1" t="s">
-        <v>1487</v>
+        <v>1486</v>
       </c>
       <c r="C744" s="2">
         <v>9234</v>
@@ -22577,7 +22577,7 @@
         <v>714908100822</v>
       </c>
       <c r="B754" s="1" t="s">
-        <v>1488</v>
+        <v>1487</v>
       </c>
       <c r="C754" s="2">
         <v>9291</v>
@@ -22669,7 +22669,7 @@
         <v>7503011998753</v>
       </c>
       <c r="B758" s="1" t="s">
-        <v>1489</v>
+        <v>1488</v>
       </c>
       <c r="C758" s="2">
         <v>9305</v>
@@ -22692,7 +22692,7 @@
         <v>7503011998760</v>
       </c>
       <c r="B759" s="1" t="s">
-        <v>1490</v>
+        <v>1489</v>
       </c>
       <c r="C759" s="2">
         <v>9306</v>
@@ -22715,7 +22715,7 @@
         <v>7503011998746</v>
       </c>
       <c r="B760" s="1" t="s">
-        <v>1491</v>
+        <v>1490</v>
       </c>
       <c r="C760" s="2">
         <v>9307</v>
@@ -22761,7 +22761,7 @@
         <v>7503000812015</v>
       </c>
       <c r="B762" s="1" t="s">
-        <v>1492</v>
+        <v>1491</v>
       </c>
       <c r="C762" s="2">
         <v>9325</v>
@@ -22876,7 +22876,7 @@
         <v>7500326106989</v>
       </c>
       <c r="B767" s="1" t="s">
-        <v>1493</v>
+        <v>1492</v>
       </c>
       <c r="C767" s="2">
         <v>9341</v>
@@ -22899,7 +22899,7 @@
         <v>7500326108747</v>
       </c>
       <c r="B768" s="1" t="s">
-        <v>1494</v>
+        <v>1493</v>
       </c>
       <c r="C768" s="2">
         <v>9343</v>
@@ -23037,7 +23037,7 @@
         <v>803288480218</v>
       </c>
       <c r="B774" s="1" t="s">
-        <v>1495</v>
+        <v>1494</v>
       </c>
       <c r="C774" s="2">
         <v>9363</v>
@@ -23060,7 +23060,7 @@
         <v>803288480737</v>
       </c>
       <c r="B775" s="1" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
       <c r="C775" s="2">
         <v>9385</v>
@@ -23129,7 +23129,7 @@
         <v>7501130704231</v>
       </c>
       <c r="B778" s="1" t="s">
-        <v>1497</v>
+        <v>1496</v>
       </c>
       <c r="C778" s="2">
         <v>9447</v>
@@ -23451,7 +23451,7 @@
         <v>631758002192</v>
       </c>
       <c r="B792" s="1" t="s">
-        <v>1498</v>
+        <v>1497</v>
       </c>
       <c r="C792" s="2">
         <v>9500</v>
@@ -23474,7 +23474,7 @@
         <v>750350000402</v>
       </c>
       <c r="B793" s="1" t="s">
-        <v>1499</v>
+        <v>1498</v>
       </c>
       <c r="C793" s="2">
         <v>9505</v>
@@ -23681,7 +23681,7 @@
         <v>7502001165489</v>
       </c>
       <c r="B802" s="1" t="s">
-        <v>1500</v>
+        <v>1499</v>
       </c>
       <c r="C802" s="2">
         <v>9594</v>
@@ -23704,7 +23704,7 @@
         <v>7501590284335</v>
       </c>
       <c r="B803" s="1" t="s">
-        <v>1501</v>
+        <v>1500</v>
       </c>
       <c r="C803" s="2">
         <v>9622</v>
@@ -23727,7 +23727,7 @@
         <v>7500462199586</v>
       </c>
       <c r="B804" s="1" t="s">
-        <v>1502</v>
+        <v>1501</v>
       </c>
       <c r="C804" s="2">
         <v>9632</v>
@@ -23750,7 +23750,7 @@
         <v>7500462199685</v>
       </c>
       <c r="B805" s="1" t="s">
-        <v>1503</v>
+        <v>1502</v>
       </c>
       <c r="C805" s="2">
         <v>9633</v>
@@ -23773,7 +23773,7 @@
         <v>7500462199692</v>
       </c>
       <c r="B806" s="1" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
       <c r="C806" s="2">
         <v>9634</v>
@@ -23865,7 +23865,7 @@
         <v>750104003574</v>
       </c>
       <c r="B810" s="1" t="s">
-        <v>1505</v>
+        <v>1504</v>
       </c>
       <c r="C810" s="2">
         <v>9704</v>
@@ -23888,7 +23888,7 @@
         <v>750104003574</v>
       </c>
       <c r="B811" s="1" t="s">
-        <v>1505</v>
+        <v>1504</v>
       </c>
       <c r="C811" s="2">
         <v>9704</v>
@@ -23911,7 +23911,7 @@
         <v>7502275940065</v>
       </c>
       <c r="B812" s="1" t="s">
-        <v>1506</v>
+        <v>1505</v>
       </c>
       <c r="C812" s="2">
         <v>9705</v>
@@ -23934,7 +23934,7 @@
         <v>750104002027</v>
       </c>
       <c r="B813" s="1" t="s">
-        <v>1507</v>
+        <v>1506</v>
       </c>
       <c r="C813" s="2">
         <v>9707</v>
@@ -23957,7 +23957,7 @@
         <v>750104003314</v>
       </c>
       <c r="B814" s="1" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="C814" s="2">
         <v>9709</v>
@@ -24003,7 +24003,7 @@
         <v>7502007700226</v>
       </c>
       <c r="B816" s="1" t="s">
-        <v>1509</v>
+        <v>1508</v>
       </c>
       <c r="C816" s="2">
         <v>9715</v>
@@ -24026,7 +24026,7 @@
         <v>7502007700271</v>
       </c>
       <c r="B817" s="1" t="s">
-        <v>1510</v>
+        <v>1509</v>
       </c>
       <c r="C817" s="2">
         <v>9716</v>
@@ -24095,7 +24095,7 @@
         <v>714908105957</v>
       </c>
       <c r="B820" s="1" t="s">
-        <v>1511</v>
+        <v>1510</v>
       </c>
       <c r="C820" s="2">
         <v>9731</v>
@@ -24118,7 +24118,7 @@
         <v>7501172018228</v>
       </c>
       <c r="B821" s="1" t="s">
-        <v>1512</v>
+        <v>1511</v>
       </c>
       <c r="C821" s="2">
         <v>9733</v>
@@ -24187,7 +24187,7 @@
         <v>7501825300885</v>
       </c>
       <c r="B824" s="1" t="s">
-        <v>1513</v>
+        <v>1512</v>
       </c>
       <c r="C824" s="2">
         <v>9737</v>
@@ -24210,7 +24210,7 @@
         <v>7503008344617</v>
       </c>
       <c r="B825" s="1" t="s">
-        <v>1514</v>
+        <v>1513</v>
       </c>
       <c r="C825" s="2">
         <v>9738</v>
@@ -24233,7 +24233,7 @@
         <v>7503002047620</v>
       </c>
       <c r="B826" s="1" t="s">
-        <v>1515</v>
+        <v>1514</v>
       </c>
       <c r="C826" s="2">
         <v>9739</v>
@@ -24279,7 +24279,7 @@
         <v>7502010840360</v>
       </c>
       <c r="B828" s="1" t="s">
-        <v>1516</v>
+        <v>1515</v>
       </c>
       <c r="C828" s="2">
         <v>9745</v>
@@ -24302,7 +24302,7 @@
         <v>7501060808016</v>
       </c>
       <c r="B829" s="1" t="s">
-        <v>1517</v>
+        <v>1516</v>
       </c>
       <c r="C829" s="2">
         <v>9747</v>
@@ -24394,7 +24394,7 @@
         <v>7502001164338</v>
       </c>
       <c r="B833" s="1" t="s">
-        <v>1518</v>
+        <v>1517</v>
       </c>
       <c r="C833" s="2">
         <v>9771</v>
@@ -24463,7 +24463,7 @@
         <v>7501258207010</v>
       </c>
       <c r="B836" s="1" t="s">
-        <v>1519</v>
+        <v>1518</v>
       </c>
       <c r="C836" s="2">
         <v>9780</v>
@@ -24509,7 +24509,7 @@
         <v>7502280810605</v>
       </c>
       <c r="B838" s="1" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
       <c r="C838" s="2">
         <v>9782</v>
@@ -24532,7 +24532,7 @@
         <v>7502280810056</v>
       </c>
       <c r="B839" s="1" t="s">
-        <v>1521</v>
+        <v>1520</v>
       </c>
       <c r="C839" s="2">
         <v>9783</v>
@@ -24831,7 +24831,7 @@
         <v>7502314550002</v>
       </c>
       <c r="B852" s="1" t="s">
-        <v>1522</v>
+        <v>1521</v>
       </c>
       <c r="C852" s="2">
         <v>9822</v>
@@ -24877,7 +24877,7 @@
         <v>7502227421666</v>
       </c>
       <c r="B854" s="1" t="s">
-        <v>1523</v>
+        <v>1522</v>
       </c>
       <c r="C854" s="2">
         <v>9842</v>
@@ -24900,7 +24900,7 @@
         <v>7500462933746</v>
       </c>
       <c r="B855" s="1" t="s">
-        <v>1524</v>
+        <v>1523</v>
       </c>
       <c r="C855" s="2">
         <v>9843</v>
@@ -25038,7 +25038,7 @@
         <v>7506021101564</v>
       </c>
       <c r="B861" s="1" t="s">
-        <v>1525</v>
+        <v>1524</v>
       </c>
       <c r="C861" s="2">
         <v>9849</v>
@@ -25084,7 +25084,7 @@
         <v>7501130711642</v>
       </c>
       <c r="B863" s="1" t="s">
-        <v>1526</v>
+        <v>1525</v>
       </c>
       <c r="C863" s="2">
         <v>9854</v>
@@ -25130,7 +25130,7 @@
         <v>750113071868</v>
       </c>
       <c r="B865" s="1" t="s">
-        <v>1527</v>
+        <v>1526</v>
       </c>
       <c r="C865" s="2">
         <v>9856</v>
@@ -25153,7 +25153,7 @@
         <v>7506021100710</v>
       </c>
       <c r="B866" s="1" t="s">
-        <v>1528</v>
+        <v>1527</v>
       </c>
       <c r="C866" s="2">
         <v>9858</v>
@@ -25245,7 +25245,7 @@
         <v>7506504900592</v>
       </c>
       <c r="B870" s="1" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="C870" s="2">
         <v>9865</v>
@@ -25268,7 +25268,7 @@
         <v>7502214018350</v>
       </c>
       <c r="B871" s="1" t="s">
-        <v>1530</v>
+        <v>1529</v>
       </c>
       <c r="C871" s="2">
         <v>9866</v>
@@ -25659,7 +25659,7 @@
         <v>759684191077</v>
       </c>
       <c r="B888" s="1" t="s">
-        <v>1531</v>
+        <v>1530</v>
       </c>
       <c r="C888" s="2">
         <v>9883</v>
@@ -26188,7 +26188,7 @@
         <v>7502259892250</v>
       </c>
       <c r="B911" s="1" t="s">
-        <v>1532</v>
+        <v>1531</v>
       </c>
       <c r="C911" s="2">
         <v>9915</v>
@@ -26487,7 +26487,7 @@
         <v>731416423427</v>
       </c>
       <c r="B924" s="1" t="s">
-        <v>1533</v>
+        <v>1532</v>
       </c>
       <c r="C924" s="2">
         <v>9928</v>
@@ -27062,7 +27062,7 @@
         <v>677144634059</v>
       </c>
       <c r="B949" s="1" t="s">
-        <v>1534</v>
+        <v>1533</v>
       </c>
       <c r="C949" s="2">
         <v>9970</v>
@@ -27085,7 +27085,7 @@
         <v>731416423427</v>
       </c>
       <c r="B950" s="1" t="s">
-        <v>1535</v>
+        <v>1534</v>
       </c>
       <c r="C950" s="2">
         <v>9971</v>
@@ -27505,7 +27505,7 @@
         <v>1143</v>
       </c>
       <c r="D968" s="2" t="s">
-        <v>1536</v>
+        <v>1535</v>
       </c>
       <c r="E968" s="13" t="s">
         <v>23</v>
@@ -27528,7 +27528,7 @@
         <v>9990</v>
       </c>
       <c r="D969" s="16" t="s">
-        <v>1537</v>
+        <v>1536</v>
       </c>
       <c r="E969" s="2" t="s">
         <v>23</v>
@@ -27551,7 +27551,7 @@
         <v>9991</v>
       </c>
       <c r="D970" s="16" t="s">
-        <v>1538</v>
+        <v>1537</v>
       </c>
       <c r="E970" s="2" t="s">
         <v>23</v>
@@ -27574,7 +27574,7 @@
         <v>9794</v>
       </c>
       <c r="D971" s="16" t="s">
-        <v>1539</v>
+        <v>1538</v>
       </c>
       <c r="E971" s="2" t="s">
         <v>23</v>
@@ -27597,7 +27597,7 @@
         <v>9992</v>
       </c>
       <c r="D972" s="16" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="E972" s="2" t="s">
         <v>23</v>
@@ -27620,7 +27620,7 @@
         <v>9993</v>
       </c>
       <c r="D973" s="16" t="s">
-        <v>1541</v>
+        <v>1540</v>
       </c>
       <c r="E973" s="2" t="s">
         <v>23</v>
@@ -27643,7 +27643,7 @@
         <v>9994</v>
       </c>
       <c r="D974" s="16" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="E974" s="2" t="s">
         <v>23</v>
@@ -27666,7 +27666,7 @@
         <v>9995</v>
       </c>
       <c r="D975" s="16" t="s">
-        <v>1543</v>
+        <v>1542</v>
       </c>
       <c r="E975" s="2" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
se agrega la 9916
</commit_message>
<xml_diff>
--- a/posiciones_buscador.xlsx
+++ b/posiciones_buscador.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\desarrollos\buscador_posiciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D990E363-5896-4BAA-B15E-FFCCA0220C7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D5F774A-2F17-4E6D-B998-8CDFCEF421F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{81345FCE-0991-44B1-AB97-4BC767A118BC}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6121" uniqueCount="1727">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6126" uniqueCount="1727">
   <si>
     <t>Cod. De Barras</t>
   </si>
@@ -5494,8 +5494,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C00A21B0-F40B-41CB-BB31-9BEA8E59BCFA}" name="Tabla13" displayName="Tabla13" ref="A1:G1002" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:G1002" xr:uid="{C00A21B0-F40B-41CB-BB31-9BEA8E59BCFA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C00A21B0-F40B-41CB-BB31-9BEA8E59BCFA}" name="Tabla13" displayName="Tabla13" ref="A1:G1003" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:G1003" xr:uid="{C00A21B0-F40B-41CB-BB31-9BEA8E59BCFA}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G967">
     <sortCondition ref="C1:C967"/>
   </sortState>
@@ -5831,7 +5831,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CD76C0E-5FFA-48DF-BC8E-37CFF7587C46}">
-  <dimension ref="A1:G1002"/>
+  <dimension ref="A1:G1003"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.90625" bestFit="1" customWidth="1"/>
@@ -28869,7 +28869,7 @@
       <c r="B1002" s="12" t="s">
         <v>999</v>
       </c>
-      <c r="C1002" s="22">
+      <c r="C1002" s="16">
         <v>1149</v>
       </c>
       <c r="D1002" s="16" t="s">
@@ -28882,13 +28882,36 @@
         <v>16</v>
       </c>
       <c r="G1002" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1003" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1003" s="20">
+        <v>7506452400038</v>
+      </c>
+      <c r="B1003" s="12" t="s">
+        <v>999</v>
+      </c>
+      <c r="C1003" s="22">
+        <v>9916</v>
+      </c>
+      <c r="D1003" s="16" t="s">
+        <v>912</v>
+      </c>
+      <c r="E1003" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1003" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1003" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="D2:D1001" calculatedColumn="1"/>
+    <ignoredError sqref="D2:D1001 D1002:D1003" calculatedColumn="1"/>
     <ignoredError sqref="B949:B950" numberStoredAsText="1"/>
   </ignoredErrors>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat: Localizador Visual v2 en paralelo (v2.html) + posiciones actualizadas
- v2.html: nueva version con croquis del almacen, ruta animada a la fila,
  rejilla anaquel x charola, escaneo por camara (HTTPS), tema claro/oscuro
  y fondo configurable. La pagina actual (index.html) queda intacta.
- posiciones_buscador.xlsx: sincronizado con la fuente de verdad local
  (la copia del repo era ~1.5h mas vieja que la ultima edicion del 24-ago).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/posiciones_buscador.xlsx
+++ b/posiciones_buscador.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\desarrollos\buscador_posiciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23D35B88-649A-4F2C-8764-42B47E0C07B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB4C1CFF-2668-4520-ABFB-54357304FAFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{81345FCE-0991-44B1-AB97-4BC767A118BC}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6177" uniqueCount="1723">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6180" uniqueCount="1723">
   <si>
     <t>Cod. De Barras</t>
   </si>
@@ -5355,7 +5355,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
@@ -5412,6 +5412,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5843,6 +5846,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="7">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{C250ABCF-3D9E-4F8C-BCD9-7F8E315ADBC3}">
+  <we:reference id="wa200010725" version="1.0.0.1" store="es-ES" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200010725" version="1.0.0.1" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;f0f9e0c3-86fa-4d24-abcf-f1482f884938&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CD76C0E-5FFA-48DF-BC8E-37CFF7587C46}">
   <dimension ref="A1:G1028"/>
@@ -20853,7 +20878,7 @@
       <c r="A653" s="9">
         <v>7502007700479</v>
       </c>
-      <c r="B653" s="9" t="s">
+      <c r="B653" s="37" t="s">
         <v>990</v>
       </c>
       <c r="C653" s="34">
@@ -20876,7 +20901,7 @@
       <c r="A654" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B654" s="9" t="s">
+      <c r="B654" s="37" t="s">
         <v>990</v>
       </c>
       <c r="C654" s="5">
@@ -20899,7 +20924,7 @@
       <c r="A655" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B655" s="9" t="s">
+      <c r="B655" s="37" t="s">
         <v>990</v>
       </c>
       <c r="C655" s="5">
@@ -21083,8 +21108,8 @@
       <c r="A663" s="1">
         <v>7501563381153</v>
       </c>
-      <c r="B663" s="1" t="e">
-        <v>#N/A</v>
+      <c r="B663" s="1" t="s">
+        <v>990</v>
       </c>
       <c r="C663" s="2">
         <v>1140</v>
@@ -21106,8 +21131,8 @@
       <c r="A664" s="1">
         <v>7506624900113</v>
       </c>
-      <c r="B664" s="1" t="e">
-        <v>#N/A</v>
+      <c r="B664" s="1" t="s">
+        <v>990</v>
       </c>
       <c r="C664" s="2">
         <v>1141</v>
@@ -21129,8 +21154,8 @@
       <c r="A665" s="1">
         <v>6934520140899</v>
       </c>
-      <c r="B665" s="1" t="e">
-        <v>#N/A</v>
+      <c r="B665" s="1" t="s">
+        <v>990</v>
       </c>
       <c r="C665" s="2">
         <v>1142</v>

</xml_diff>